<commit_message>
First commit entire project pushing for first time
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestDataSheet.xlsx
+++ b/src/test/resources/testdata/TestDataSheet.xlsx
@@ -1,32 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AzeemK\eclipse-workspace\TestingMiniBytesFramework\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AzeemK\eclipse-workspace\Document_Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F234B741-846B-4A14-B9FF-76C0B24E0CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4417E5-A06F-40EF-9148-7299F4FD1102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RunManager" sheetId="3" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="92">
   <si>
     <t>Username</t>
   </si>
@@ -160,9 +171,6 @@
     <t>Martinez</t>
   </si>
   <si>
-    <t>Admin</t>
-  </si>
-  <si>
     <t>TestMethodName</t>
   </si>
   <si>
@@ -178,67 +186,133 @@
     <t>InvocationCount</t>
   </si>
   <si>
-    <t>validloginTest</t>
-  </si>
-  <si>
-    <t>inValidloginTest1</t>
-  </si>
-  <si>
-    <t>inValidloginTest2</t>
-  </si>
-  <si>
-    <t>inValidloginTest3</t>
-  </si>
-  <si>
-    <t>To Verify Login with Invalid Username &amp; Password</t>
-  </si>
-  <si>
     <t>yes</t>
   </si>
   <si>
-    <t>To Verify Login with valid username &amp; Invalid Password</t>
-  </si>
-  <si>
-    <t>To Verify Login with InValid username &amp; Valid Password</t>
-  </si>
-  <si>
     <t>Aadmin</t>
   </si>
   <si>
     <t>TC-ID</t>
   </si>
   <si>
-    <t>LOGIN_AUTO_TC_001</t>
-  </si>
-  <si>
-    <t>LOGIN_AUTO_TC_002</t>
-  </si>
-  <si>
-    <t>LOGIN_AUTO_TC_003</t>
-  </si>
-  <si>
-    <t>LOGIN_AUTO_TC_004</t>
-  </si>
-  <si>
     <t>Browser</t>
   </si>
   <si>
     <t>chrome</t>
   </si>
   <si>
-    <t>firefox</t>
-  </si>
-  <si>
-    <t>To Validate the Login with Valid UserName &amp; Password</t>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>QWRtaW5AMTIz</t>
+  </si>
+  <si>
+    <t>ValidLoginTest</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>verifyUIElements</t>
+  </si>
+  <si>
+    <t>Verify all the UI Element in the Landing Page.</t>
+  </si>
+  <si>
+    <t>TC_001</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>Validate the User Login with Valid Username &amp; Password</t>
+  </si>
+  <si>
+    <t>Validate the User Login with valid username &amp; Invalid Password</t>
+  </si>
+  <si>
+    <t>Validate the User Login with invalid username &amp; valid Password</t>
+  </si>
+  <si>
+    <t>Validate the User Login with invalid username &amp; Password</t>
+  </si>
+  <si>
+    <t>InvalidPassword</t>
+  </si>
+  <si>
+    <t>Invalidname</t>
+  </si>
+  <si>
+    <t>InvalidUP</t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>InvalidPasswordLength</t>
+  </si>
+  <si>
+    <t>Validate the User Login with invalid Password length</t>
+  </si>
+  <si>
+    <t>QWRtaW4=</t>
+  </si>
+  <si>
+    <t>QWRtaW5AMTI0</t>
   </si>
   <si>
     <t>no</t>
   </si>
   <si>
-    <t>YWRtaW4xMjM=</t>
-  </si>
-  <si>
-    <t>YWRtaW4=</t>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>CreateDomain</t>
+  </si>
+  <si>
+    <t>Validate Domain Creation</t>
+  </si>
+  <si>
+    <t>Domain Name</t>
+  </si>
+  <si>
+    <t>Automation Test</t>
+  </si>
+  <si>
+    <t>Domain Description</t>
+  </si>
+  <si>
+    <t>Testing Domain Creation via Automation</t>
+  </si>
+  <si>
+    <t>ValidLogin_SignOutTest</t>
+  </si>
+  <si>
+    <t>Valid Login &amp; Logout Test</t>
+  </si>
+  <si>
+    <t>ValidateDeleteDomain</t>
+  </si>
+  <si>
+    <t>TC_008</t>
+  </si>
+  <si>
+    <t>TC_009</t>
+  </si>
+  <si>
+    <t>Validate Delete Domain Functionality</t>
+  </si>
+  <si>
+    <t>Unloading</t>
   </si>
 </sst>
 </file>
@@ -290,10 +364,36 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -302,7 +402,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -310,14 +410,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -599,162 +708,370 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D86C8E9-5594-4343-AC78-84D4D9B42719}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="58.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="D2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3">
+        <v>1</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="3">
+        <v>1</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="B6" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
+      <c r="G6" s="3">
+        <v>1</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1</v>
+      </c>
+      <c r="G7" s="3">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="H1" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="E8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3">
+        <v>1</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" s="3">
+        <v>1</v>
+      </c>
+      <c r="G9" s="3">
+        <v>1</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="3">
-        <v>1</v>
-      </c>
-      <c r="G2" s="3">
-        <v>1</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" s="3">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3">
-        <v>1</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3">
-        <v>1</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="J9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F5" s="3">
-        <v>1</v>
-      </c>
-      <c r="G5" s="3">
-        <v>1</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>70</v>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
+      <c r="G10" s="3">
+        <v>1</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>